<commit_message>
Add SharePoint/OneDrive cloud script and register starter rows
- Build-SharePoint-Library.ps1: provisions the same coded folder tree
  directly in a SharePoint Online / OneDrive-for-Business document
  library via PnP PowerShell (idempotent)
- File register: add 11 starter template rows, one per category, showing
  the naming convention in context; force recalc-on-load
- README: document cloud setup options and starter rows

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Q5wApasUKcoyLKa16oUzQ3
</commit_message>
<xml_diff>
--- a/file-organization-system/Alhasa-Palm-HSE-File-Register.xlsx
+++ b/file-organization-system/Alhasa-Palm-HSE-File-Register.xlsx
@@ -1027,7 +1027,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J304"/>
+  <dimension ref="A1:J314"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -1111,174 +1111,574 @@
     <row r="4">
       <c r="A4" s="13" t="inlineStr">
         <is>
+          <t>APP-PM-MOM-001-20260705-R0_HSE-Kickoff-Meeting-Minutes</t>
+        </is>
+      </c>
+      <c r="B4" s="13" t="inlineStr">
+        <is>
+          <t>PM</t>
+        </is>
+      </c>
+      <c r="C4" s="13" t="inlineStr">
+        <is>
+          <t>MOM</t>
+        </is>
+      </c>
+      <c r="D4" s="14" t="inlineStr">
+        <is>
+          <t>HSE kickoff meeting minutes</t>
+        </is>
+      </c>
+      <c r="E4" s="13" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="F4" s="13" t="inlineStr">
+        <is>
+          <t>R0</t>
+        </is>
+      </c>
+      <c r="G4" s="13" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="H4" s="13" t="inlineStr">
+        <is>
+          <t>M. Alshehri</t>
+        </is>
+      </c>
+      <c r="I4" s="14" t="inlineStr">
+        <is>
+          <t>00_PM\00-04_Meeting-Minutes</t>
+        </is>
+      </c>
+      <c r="J4" s="14" t="inlineStr">
+        <is>
+          <t>TEMPLATE - edit or delete</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="13" t="inlineStr">
+        <is>
+          <t>APP-HSE-MS-002-20260601-R1_Excavation-Method-Statement</t>
+        </is>
+      </c>
+      <c r="B5" s="13" t="inlineStr">
+        <is>
+          <t>HSE</t>
+        </is>
+      </c>
+      <c r="C5" s="13" t="inlineStr">
+        <is>
+          <t>MS</t>
+        </is>
+      </c>
+      <c r="D5" s="14" t="inlineStr">
+        <is>
+          <t>Method statement - excavation works</t>
+        </is>
+      </c>
+      <c r="E5" s="13" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="F5" s="13" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="G5" s="13" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="H5" s="13" t="inlineStr">
+        <is>
+          <t>HSE Manager</t>
+        </is>
+      </c>
+      <c r="I5" s="14" t="inlineStr">
+        <is>
+          <t>10_HSE\10-02_Method-Statements</t>
+        </is>
+      </c>
+      <c r="J5" s="14" t="inlineStr">
+        <is>
+          <t>TEMPLATE - edit or delete</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="13" t="inlineStr">
+        <is>
+          <t>APP-PTW-PMT-045-20260718-R0_HotWork-ZoneB</t>
+        </is>
+      </c>
+      <c r="B6" s="13" t="inlineStr">
+        <is>
+          <t>PTW</t>
+        </is>
+      </c>
+      <c r="C6" s="13" t="inlineStr">
+        <is>
+          <t>PMT</t>
+        </is>
+      </c>
+      <c r="D6" s="14" t="inlineStr">
+        <is>
+          <t>Hot work permit - welding at Zone B</t>
+        </is>
+      </c>
+      <c r="E6" s="13" t="inlineStr">
+        <is>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="F6" s="13" t="inlineStr">
+        <is>
+          <t>R0</t>
+        </is>
+      </c>
+      <c r="G6" s="13" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="H6" s="13" t="inlineStr">
+        <is>
+          <t>Site Supervisor</t>
+        </is>
+      </c>
+      <c r="I6" s="14" t="inlineStr">
+        <is>
+          <t>20_PTW\20-01_Hot-Work</t>
+        </is>
+      </c>
+      <c r="J6" s="14" t="inlineStr">
+        <is>
+          <t>TEMPLATE - edit or delete</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="13" t="inlineStr">
+        <is>
           <t>APP-INC-INV-001-20260715-R0_Scaffold-Fall-NearMiss</t>
         </is>
       </c>
-      <c r="B4" s="13" t="inlineStr">
+      <c r="B7" s="13" t="inlineStr">
         <is>
           <t>INC</t>
         </is>
       </c>
-      <c r="C4" s="13" t="inlineStr">
+      <c r="C7" s="13" t="inlineStr">
         <is>
           <t>INV</t>
         </is>
       </c>
-      <c r="D4" s="14" t="inlineStr">
+      <c r="D7" s="14" t="inlineStr">
         <is>
           <t>Investigation report - scaffold fall near-miss at Zone B</t>
         </is>
       </c>
-      <c r="E4" s="13" t="inlineStr">
+      <c r="E7" s="13" t="inlineStr">
         <is>
           <t>2026-07-15</t>
         </is>
       </c>
-      <c r="F4" s="13" t="inlineStr">
+      <c r="F7" s="13" t="inlineStr">
         <is>
           <t>R0</t>
         </is>
       </c>
-      <c r="G4" s="13" t="inlineStr">
+      <c r="G7" s="13" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="H4" s="13" t="inlineStr">
+      <c r="H7" s="13" t="inlineStr">
         <is>
           <t>M. Alshehri</t>
         </is>
       </c>
-      <c r="I4" s="14" t="inlineStr">
+      <c r="I7" s="14" t="inlineStr">
         <is>
           <t>30_INC\30-02_Investigations-and-RCA</t>
         </is>
       </c>
-      <c r="J4" s="14" t="inlineStr">
-        <is>
-          <t>Example row - replace with your data</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="15" t="n"/>
-      <c r="B5" s="15" t="n"/>
-      <c r="C5" s="15" t="n"/>
-      <c r="D5" s="16" t="n"/>
-      <c r="E5" s="15" t="n"/>
-      <c r="F5" s="15" t="n"/>
-      <c r="G5" s="15" t="n"/>
-      <c r="H5" s="15" t="n"/>
-      <c r="I5" s="16" t="n"/>
-      <c r="J5" s="16" t="n"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="17" t="n"/>
-      <c r="B6" s="17" t="n"/>
-      <c r="C6" s="17" t="n"/>
-      <c r="D6" s="18" t="n"/>
-      <c r="E6" s="17" t="n"/>
-      <c r="F6" s="17" t="n"/>
-      <c r="G6" s="17" t="n"/>
-      <c r="H6" s="17" t="n"/>
-      <c r="I6" s="18" t="n"/>
-      <c r="J6" s="18" t="n"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="15" t="n"/>
-      <c r="B7" s="15" t="n"/>
-      <c r="C7" s="15" t="n"/>
-      <c r="D7" s="16" t="n"/>
-      <c r="E7" s="15" t="n"/>
-      <c r="F7" s="15" t="n"/>
-      <c r="G7" s="15" t="n"/>
-      <c r="H7" s="15" t="n"/>
-      <c r="I7" s="16" t="n"/>
-      <c r="J7" s="16" t="n"/>
+      <c r="J7" s="14" t="inlineStr">
+        <is>
+          <t>TEMPLATE - edit or delete</t>
+        </is>
+      </c>
     </row>
     <row r="8">
-      <c r="A8" s="17" t="n"/>
-      <c r="B8" s="17" t="n"/>
-      <c r="C8" s="17" t="n"/>
-      <c r="D8" s="18" t="n"/>
-      <c r="E8" s="17" t="n"/>
-      <c r="F8" s="17" t="n"/>
-      <c r="G8" s="17" t="n"/>
-      <c r="H8" s="17" t="n"/>
-      <c r="I8" s="18" t="n"/>
-      <c r="J8" s="18" t="n"/>
+      <c r="A8" s="13" t="inlineStr">
+        <is>
+          <t>APP-OBS-RPT-012-20260719-R0_Unsafe-Housekeeping-GateA</t>
+        </is>
+      </c>
+      <c r="B8" s="13" t="inlineStr">
+        <is>
+          <t>OBS</t>
+        </is>
+      </c>
+      <c r="C8" s="13" t="inlineStr">
+        <is>
+          <t>RPT</t>
+        </is>
+      </c>
+      <c r="D8" s="14" t="inlineStr">
+        <is>
+          <t>Safety observation - poor housekeeping at Gate A</t>
+        </is>
+      </c>
+      <c r="E8" s="13" t="inlineStr">
+        <is>
+          <t>2026-07-19</t>
+        </is>
+      </c>
+      <c r="F8" s="13" t="inlineStr">
+        <is>
+          <t>R0</t>
+        </is>
+      </c>
+      <c r="G8" s="13" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="H8" s="13" t="inlineStr">
+        <is>
+          <t>HSE Officer</t>
+        </is>
+      </c>
+      <c r="I8" s="14" t="inlineStr">
+        <is>
+          <t>40_OBS\40-01_Safety-Observations</t>
+        </is>
+      </c>
+      <c r="J8" s="14" t="inlineStr">
+        <is>
+          <t>TEMPLATE - edit or delete</t>
+        </is>
+      </c>
     </row>
     <row r="9">
-      <c r="A9" s="15" t="n"/>
-      <c r="B9" s="15" t="n"/>
-      <c r="C9" s="15" t="n"/>
-      <c r="D9" s="16" t="n"/>
-      <c r="E9" s="15" t="n"/>
-      <c r="F9" s="15" t="n"/>
-      <c r="G9" s="15" t="n"/>
-      <c r="H9" s="15" t="n"/>
-      <c r="I9" s="16" t="n"/>
-      <c r="J9" s="16" t="n"/>
+      <c r="A9" s="13" t="inlineStr">
+        <is>
+          <t>APP-TRN-CERT-030-20260610-R0_Ali-Hassan-Confined-Space</t>
+        </is>
+      </c>
+      <c r="B9" s="13" t="inlineStr">
+        <is>
+          <t>TRN</t>
+        </is>
+      </c>
+      <c r="C9" s="13" t="inlineStr">
+        <is>
+          <t>CERT</t>
+        </is>
+      </c>
+      <c r="D9" s="14" t="inlineStr">
+        <is>
+          <t>Confined space entry certificate - Ali Hassan</t>
+        </is>
+      </c>
+      <c r="E9" s="13" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="F9" s="13" t="inlineStr">
+        <is>
+          <t>R0</t>
+        </is>
+      </c>
+      <c r="G9" s="13" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="H9" s="13" t="inlineStr">
+        <is>
+          <t>Training Coord.</t>
+        </is>
+      </c>
+      <c r="I9" s="14" t="inlineStr">
+        <is>
+          <t>50_TRN\50-02_Competency-Certificates</t>
+        </is>
+      </c>
+      <c r="J9" s="14" t="inlineStr">
+        <is>
+          <t>TEMPLATE - edit or delete</t>
+        </is>
+      </c>
     </row>
     <row r="10">
-      <c r="A10" s="17" t="n"/>
-      <c r="B10" s="17" t="n"/>
-      <c r="C10" s="17" t="n"/>
-      <c r="D10" s="18" t="n"/>
-      <c r="E10" s="17" t="n"/>
-      <c r="F10" s="17" t="n"/>
-      <c r="G10" s="17" t="n"/>
-      <c r="H10" s="17" t="n"/>
-      <c r="I10" s="18" t="n"/>
-      <c r="J10" s="18" t="n"/>
+      <c r="A10" s="13" t="inlineStr">
+        <is>
+          <t>APP-CRT-CERT-008-20260620-R0_Crane-Annual-Third-Party</t>
+        </is>
+      </c>
+      <c r="B10" s="13" t="inlineStr">
+        <is>
+          <t>CRT</t>
+        </is>
+      </c>
+      <c r="C10" s="13" t="inlineStr">
+        <is>
+          <t>CERT</t>
+        </is>
+      </c>
+      <c r="D10" s="14" t="inlineStr">
+        <is>
+          <t>Third-party annual inspection certificate - mobile crane</t>
+        </is>
+      </c>
+      <c r="E10" s="13" t="inlineStr">
+        <is>
+          <t>2026-06-20</t>
+        </is>
+      </c>
+      <c r="F10" s="13" t="inlineStr">
+        <is>
+          <t>R0</t>
+        </is>
+      </c>
+      <c r="G10" s="13" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="H10" s="13" t="inlineStr">
+        <is>
+          <t>Plant Dept.</t>
+        </is>
+      </c>
+      <c r="I10" s="14" t="inlineStr">
+        <is>
+          <t>60_CRT\60-02_Third-Party-Inspections</t>
+        </is>
+      </c>
+      <c r="J10" s="14" t="inlineStr">
+        <is>
+          <t>TEMPLATE - edit or delete</t>
+        </is>
+      </c>
     </row>
     <row r="11">
-      <c r="A11" s="15" t="n"/>
-      <c r="B11" s="15" t="n"/>
-      <c r="C11" s="15" t="n"/>
-      <c r="D11" s="16" t="n"/>
-      <c r="E11" s="15" t="n"/>
-      <c r="F11" s="15" t="n"/>
-      <c r="G11" s="15" t="n"/>
-      <c r="H11" s="15" t="n"/>
-      <c r="I11" s="16" t="n"/>
-      <c r="J11" s="16" t="n"/>
+      <c r="A11" s="13" t="inlineStr">
+        <is>
+          <t>APP-RPT-RPT-006-20260701-R1_Monthly-HSE-Report-Jun2026</t>
+        </is>
+      </c>
+      <c r="B11" s="13" t="inlineStr">
+        <is>
+          <t>RPT</t>
+        </is>
+      </c>
+      <c r="C11" s="13" t="inlineStr">
+        <is>
+          <t>RPT</t>
+        </is>
+      </c>
+      <c r="D11" s="14" t="inlineStr">
+        <is>
+          <t>Monthly HSE performance report - June 2026</t>
+        </is>
+      </c>
+      <c r="E11" s="13" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="F11" s="13" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="G11" s="13" t="inlineStr">
+        <is>
+          <t>Approved</t>
+        </is>
+      </c>
+      <c r="H11" s="13" t="inlineStr">
+        <is>
+          <t>M. Alshehri</t>
+        </is>
+      </c>
+      <c r="I11" s="14" t="inlineStr">
+        <is>
+          <t>70_RPT\70-03_Monthly-HSE-Reports</t>
+        </is>
+      </c>
+      <c r="J11" s="14" t="inlineStr">
+        <is>
+          <t>TEMPLATE - edit or delete</t>
+        </is>
+      </c>
     </row>
     <row r="12">
-      <c r="A12" s="17" t="n"/>
-      <c r="B12" s="17" t="n"/>
-      <c r="C12" s="17" t="n"/>
-      <c r="D12" s="18" t="n"/>
-      <c r="E12" s="17" t="n"/>
-      <c r="F12" s="17" t="n"/>
-      <c r="G12" s="17" t="n"/>
-      <c r="H12" s="17" t="n"/>
-      <c r="I12" s="18" t="n"/>
-      <c r="J12" s="18" t="n"/>
+      <c r="A12" s="13" t="inlineStr">
+        <is>
+          <t>APP-MED-PHO-014-20260719-R0_GateA-Housekeeping-Photo</t>
+        </is>
+      </c>
+      <c r="B12" s="13" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="C12" s="13" t="inlineStr">
+        <is>
+          <t>PHO</t>
+        </is>
+      </c>
+      <c r="D12" s="14" t="inlineStr">
+        <is>
+          <t>Photo - Gate A housekeeping (linked to OBS-012)</t>
+        </is>
+      </c>
+      <c r="E12" s="13" t="inlineStr">
+        <is>
+          <t>2026-07-19</t>
+        </is>
+      </c>
+      <c r="F12" s="13" t="inlineStr">
+        <is>
+          <t>R0</t>
+        </is>
+      </c>
+      <c r="G12" s="13" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="H12" s="13" t="inlineStr">
+        <is>
+          <t>HSE Officer</t>
+        </is>
+      </c>
+      <c r="I12" s="14" t="inlineStr">
+        <is>
+          <t>80_MED\80-04_Observation-Photos</t>
+        </is>
+      </c>
+      <c r="J12" s="14" t="inlineStr">
+        <is>
+          <t>TEMPLATE - edit or delete</t>
+        </is>
+      </c>
     </row>
     <row r="13">
-      <c r="A13" s="15" t="n"/>
-      <c r="B13" s="15" t="n"/>
-      <c r="C13" s="15" t="n"/>
-      <c r="D13" s="16" t="n"/>
-      <c r="E13" s="15" t="n"/>
-      <c r="F13" s="15" t="n"/>
-      <c r="G13" s="15" t="n"/>
-      <c r="H13" s="15" t="n"/>
-      <c r="I13" s="16" t="n"/>
-      <c r="J13" s="16" t="n"/>
+      <c r="A13" s="13" t="inlineStr">
+        <is>
+          <t>APP-DWG-PLN-003-20260515-R0_Site-Layout-PhaseB</t>
+        </is>
+      </c>
+      <c r="B13" s="13" t="inlineStr">
+        <is>
+          <t>DWG</t>
+        </is>
+      </c>
+      <c r="C13" s="13" t="inlineStr">
+        <is>
+          <t>PLN</t>
+        </is>
+      </c>
+      <c r="D13" s="14" t="inlineStr">
+        <is>
+          <t>Site layout drawing - Phase B</t>
+        </is>
+      </c>
+      <c r="E13" s="13" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="F13" s="13" t="inlineStr">
+        <is>
+          <t>R0</t>
+        </is>
+      </c>
+      <c r="G13" s="13" t="inlineStr">
+        <is>
+          <t>For Review</t>
+        </is>
+      </c>
+      <c r="H13" s="13" t="inlineStr">
+        <is>
+          <t>Engineering</t>
+        </is>
+      </c>
+      <c r="I13" s="14" t="inlineStr">
+        <is>
+          <t>90_DWG\90-01_Site-Layout-and-Maps</t>
+        </is>
+      </c>
+      <c r="J13" s="14" t="inlineStr">
+        <is>
+          <t>TEMPLATE - edit or delete</t>
+        </is>
+      </c>
     </row>
     <row r="14">
-      <c r="A14" s="17" t="n"/>
-      <c r="B14" s="17" t="n"/>
-      <c r="C14" s="17" t="n"/>
-      <c r="D14" s="18" t="n"/>
-      <c r="E14" s="17" t="n"/>
-      <c r="F14" s="17" t="n"/>
-      <c r="G14" s="17" t="n"/>
-      <c r="H14" s="17" t="n"/>
-      <c r="I14" s="18" t="n"/>
-      <c r="J14" s="18" t="n"/>
+      <c r="A14" s="13" t="inlineStr">
+        <is>
+          <t>APP-ARC-RPT-002-20250101-R0_2025-Closed-HSE-Report</t>
+        </is>
+      </c>
+      <c r="B14" s="13" t="inlineStr">
+        <is>
+          <t>ARC</t>
+        </is>
+      </c>
+      <c r="C14" s="13" t="inlineStr">
+        <is>
+          <t>RPT</t>
+        </is>
+      </c>
+      <c r="D14" s="14" t="inlineStr">
+        <is>
+          <t>Archived closed HSE report - 2025</t>
+        </is>
+      </c>
+      <c r="E14" s="13" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="F14" s="13" t="inlineStr">
+        <is>
+          <t>R0</t>
+        </is>
+      </c>
+      <c r="G14" s="13" t="inlineStr">
+        <is>
+          <t>Superseded</t>
+        </is>
+      </c>
+      <c r="H14" s="13" t="inlineStr">
+        <is>
+          <t>Document Control</t>
+        </is>
+      </c>
+      <c r="I14" s="14" t="inlineStr">
+        <is>
+          <t>99_ARC\99-02_Closed-Records</t>
+        </is>
+      </c>
+      <c r="J14" s="14" t="inlineStr">
+        <is>
+          <t>TEMPLATE - edit or delete</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="15" t="n"/>
@@ -4760,19 +5160,139 @@
       <c r="I304" s="18" t="n"/>
       <c r="J304" s="18" t="n"/>
     </row>
+    <row r="305">
+      <c r="A305" s="15" t="n"/>
+      <c r="B305" s="15" t="n"/>
+      <c r="C305" s="15" t="n"/>
+      <c r="D305" s="16" t="n"/>
+      <c r="E305" s="15" t="n"/>
+      <c r="F305" s="15" t="n"/>
+      <c r="G305" s="15" t="n"/>
+      <c r="H305" s="15" t="n"/>
+      <c r="I305" s="16" t="n"/>
+      <c r="J305" s="16" t="n"/>
+    </row>
+    <row r="306">
+      <c r="A306" s="17" t="n"/>
+      <c r="B306" s="17" t="n"/>
+      <c r="C306" s="17" t="n"/>
+      <c r="D306" s="18" t="n"/>
+      <c r="E306" s="17" t="n"/>
+      <c r="F306" s="17" t="n"/>
+      <c r="G306" s="17" t="n"/>
+      <c r="H306" s="17" t="n"/>
+      <c r="I306" s="18" t="n"/>
+      <c r="J306" s="18" t="n"/>
+    </row>
+    <row r="307">
+      <c r="A307" s="15" t="n"/>
+      <c r="B307" s="15" t="n"/>
+      <c r="C307" s="15" t="n"/>
+      <c r="D307" s="16" t="n"/>
+      <c r="E307" s="15" t="n"/>
+      <c r="F307" s="15" t="n"/>
+      <c r="G307" s="15" t="n"/>
+      <c r="H307" s="15" t="n"/>
+      <c r="I307" s="16" t="n"/>
+      <c r="J307" s="16" t="n"/>
+    </row>
+    <row r="308">
+      <c r="A308" s="17" t="n"/>
+      <c r="B308" s="17" t="n"/>
+      <c r="C308" s="17" t="n"/>
+      <c r="D308" s="18" t="n"/>
+      <c r="E308" s="17" t="n"/>
+      <c r="F308" s="17" t="n"/>
+      <c r="G308" s="17" t="n"/>
+      <c r="H308" s="17" t="n"/>
+      <c r="I308" s="18" t="n"/>
+      <c r="J308" s="18" t="n"/>
+    </row>
+    <row r="309">
+      <c r="A309" s="15" t="n"/>
+      <c r="B309" s="15" t="n"/>
+      <c r="C309" s="15" t="n"/>
+      <c r="D309" s="16" t="n"/>
+      <c r="E309" s="15" t="n"/>
+      <c r="F309" s="15" t="n"/>
+      <c r="G309" s="15" t="n"/>
+      <c r="H309" s="15" t="n"/>
+      <c r="I309" s="16" t="n"/>
+      <c r="J309" s="16" t="n"/>
+    </row>
+    <row r="310">
+      <c r="A310" s="17" t="n"/>
+      <c r="B310" s="17" t="n"/>
+      <c r="C310" s="17" t="n"/>
+      <c r="D310" s="18" t="n"/>
+      <c r="E310" s="17" t="n"/>
+      <c r="F310" s="17" t="n"/>
+      <c r="G310" s="17" t="n"/>
+      <c r="H310" s="17" t="n"/>
+      <c r="I310" s="18" t="n"/>
+      <c r="J310" s="18" t="n"/>
+    </row>
+    <row r="311">
+      <c r="A311" s="15" t="n"/>
+      <c r="B311" s="15" t="n"/>
+      <c r="C311" s="15" t="n"/>
+      <c r="D311" s="16" t="n"/>
+      <c r="E311" s="15" t="n"/>
+      <c r="F311" s="15" t="n"/>
+      <c r="G311" s="15" t="n"/>
+      <c r="H311" s="15" t="n"/>
+      <c r="I311" s="16" t="n"/>
+      <c r="J311" s="16" t="n"/>
+    </row>
+    <row r="312">
+      <c r="A312" s="17" t="n"/>
+      <c r="B312" s="17" t="n"/>
+      <c r="C312" s="17" t="n"/>
+      <c r="D312" s="18" t="n"/>
+      <c r="E312" s="17" t="n"/>
+      <c r="F312" s="17" t="n"/>
+      <c r="G312" s="17" t="n"/>
+      <c r="H312" s="17" t="n"/>
+      <c r="I312" s="18" t="n"/>
+      <c r="J312" s="18" t="n"/>
+    </row>
+    <row r="313">
+      <c r="A313" s="15" t="n"/>
+      <c r="B313" s="15" t="n"/>
+      <c r="C313" s="15" t="n"/>
+      <c r="D313" s="16" t="n"/>
+      <c r="E313" s="15" t="n"/>
+      <c r="F313" s="15" t="n"/>
+      <c r="G313" s="15" t="n"/>
+      <c r="H313" s="15" t="n"/>
+      <c r="I313" s="16" t="n"/>
+      <c r="J313" s="16" t="n"/>
+    </row>
+    <row r="314">
+      <c r="A314" s="17" t="n"/>
+      <c r="B314" s="17" t="n"/>
+      <c r="C314" s="17" t="n"/>
+      <c r="D314" s="18" t="n"/>
+      <c r="E314" s="17" t="n"/>
+      <c r="F314" s="17" t="n"/>
+      <c r="G314" s="17" t="n"/>
+      <c r="H314" s="17" t="n"/>
+      <c r="I314" s="18" t="n"/>
+      <c r="J314" s="18" t="n"/>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:J1"/>
     <mergeCell ref="A2:J2"/>
   </mergeCells>
   <dataValidations count="3">
-    <dataValidation sqref="B4:B304" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="B4:B314" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"PM,HSE,PTW,INC,OBS,TRN,CRT,RPT,MED,DWG,ARC"</formula1>
     </dataValidation>
-    <dataValidation sqref="C4:C304" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="C4:C314" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"RPT,FRM,CHK,PMT,CERT,MOM,LTR,RA,MS,INV,PHO,LOG,PLN,PRO,TBT,AUD"</formula1>
     </dataValidation>
-    <dataValidation sqref="G4:G304" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G4:G314" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Open,In Progress,Closed,Approved,Superseded,For Review"</formula1>
     </dataValidation>
   </dataValidations>
@@ -4808,7 +5328,7 @@
         </is>
       </c>
       <c r="C4" s="21">
-        <f>COUNTA('File Register'!A4:A304)-1</f>
+        <f>COUNTA('File Register'!A4:A314)</f>
         <v/>
       </c>
     </row>
@@ -4827,7 +5347,7 @@
         </is>
       </c>
       <c r="C7" s="22">
-        <f>COUNTIF('File Register'!$B$4:$B$304,B7)</f>
+        <f>COUNTIF('File Register'!$B$4:$B$314,B7)</f>
         <v/>
       </c>
     </row>
@@ -4838,7 +5358,7 @@
         </is>
       </c>
       <c r="C8" s="22">
-        <f>COUNTIF('File Register'!$B$4:$B$304,B8)</f>
+        <f>COUNTIF('File Register'!$B$4:$B$314,B8)</f>
         <v/>
       </c>
     </row>
@@ -4849,7 +5369,7 @@
         </is>
       </c>
       <c r="C9" s="22">
-        <f>COUNTIF('File Register'!$B$4:$B$304,B9)</f>
+        <f>COUNTIF('File Register'!$B$4:$B$314,B9)</f>
         <v/>
       </c>
     </row>
@@ -4860,7 +5380,7 @@
         </is>
       </c>
       <c r="C10" s="22">
-        <f>COUNTIF('File Register'!$B$4:$B$304,B10)</f>
+        <f>COUNTIF('File Register'!$B$4:$B$314,B10)</f>
         <v/>
       </c>
     </row>
@@ -4871,7 +5391,7 @@
         </is>
       </c>
       <c r="C11" s="22">
-        <f>COUNTIF('File Register'!$B$4:$B$304,B11)</f>
+        <f>COUNTIF('File Register'!$B$4:$B$314,B11)</f>
         <v/>
       </c>
     </row>
@@ -4882,7 +5402,7 @@
         </is>
       </c>
       <c r="C12" s="22">
-        <f>COUNTIF('File Register'!$B$4:$B$304,B12)</f>
+        <f>COUNTIF('File Register'!$B$4:$B$314,B12)</f>
         <v/>
       </c>
     </row>
@@ -4893,7 +5413,7 @@
         </is>
       </c>
       <c r="C13" s="22">
-        <f>COUNTIF('File Register'!$B$4:$B$304,B13)</f>
+        <f>COUNTIF('File Register'!$B$4:$B$314,B13)</f>
         <v/>
       </c>
     </row>
@@ -4904,7 +5424,7 @@
         </is>
       </c>
       <c r="C14" s="22">
-        <f>COUNTIF('File Register'!$B$4:$B$304,B14)</f>
+        <f>COUNTIF('File Register'!$B$4:$B$314,B14)</f>
         <v/>
       </c>
     </row>
@@ -4915,7 +5435,7 @@
         </is>
       </c>
       <c r="C15" s="22">
-        <f>COUNTIF('File Register'!$B$4:$B$304,B15)</f>
+        <f>COUNTIF('File Register'!$B$4:$B$314,B15)</f>
         <v/>
       </c>
     </row>
@@ -4926,7 +5446,7 @@
         </is>
       </c>
       <c r="C16" s="22">
-        <f>COUNTIF('File Register'!$B$4:$B$304,B16)</f>
+        <f>COUNTIF('File Register'!$B$4:$B$314,B16)</f>
         <v/>
       </c>
     </row>
@@ -4937,7 +5457,7 @@
         </is>
       </c>
       <c r="C17" s="22">
-        <f>COUNTIF('File Register'!$B$4:$B$304,B17)</f>
+        <f>COUNTIF('File Register'!$B$4:$B$314,B17)</f>
         <v/>
       </c>
     </row>
@@ -4956,7 +5476,7 @@
         </is>
       </c>
       <c r="C20" s="22">
-        <f>COUNTIF('File Register'!$G$4:$G$304,B20)</f>
+        <f>COUNTIF('File Register'!$G$4:$G$314,B20)</f>
         <v/>
       </c>
     </row>
@@ -4967,7 +5487,7 @@
         </is>
       </c>
       <c r="C21" s="22">
-        <f>COUNTIF('File Register'!$G$4:$G$304,B21)</f>
+        <f>COUNTIF('File Register'!$G$4:$G$314,B21)</f>
         <v/>
       </c>
     </row>
@@ -4978,7 +5498,7 @@
         </is>
       </c>
       <c r="C22" s="22">
-        <f>COUNTIF('File Register'!$G$4:$G$304,B22)</f>
+        <f>COUNTIF('File Register'!$G$4:$G$314,B22)</f>
         <v/>
       </c>
     </row>
@@ -4989,7 +5509,7 @@
         </is>
       </c>
       <c r="C23" s="22">
-        <f>COUNTIF('File Register'!$G$4:$G$304,B23)</f>
+        <f>COUNTIF('File Register'!$G$4:$G$314,B23)</f>
         <v/>
       </c>
     </row>
@@ -5000,7 +5520,7 @@
         </is>
       </c>
       <c r="C24" s="22">
-        <f>COUNTIF('File Register'!$G$4:$G$304,B24)</f>
+        <f>COUNTIF('File Register'!$G$4:$G$314,B24)</f>
         <v/>
       </c>
     </row>
@@ -5011,7 +5531,7 @@
         </is>
       </c>
       <c r="C25" s="22">
-        <f>COUNTIF('File Register'!$G$4:$G$304,B25)</f>
+        <f>COUNTIF('File Register'!$G$4:$G$314,B25)</f>
         <v/>
       </c>
     </row>

</xml_diff>